<commit_message>
feat: add M-script assets and implement relative path architecture
- Exported Power Query logic to /powerquery as standalone .m files.
- Implemented ProjectPath parameter logic for office/home portability.
- Standardized Excel mapping sources to use 'Sheet1' and professional headers.
- Updated README.md to reflect the new dynamic mapping architecture.
</commit_message>
<xml_diff>
--- a/docs/Uniconta_Labels_Custom.xlsx
+++ b/docs/Uniconta_Labels_Custom.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eilersenelectric-my.sharepoint.com/personal/vnn_eilersen_com/Documents/Dokumenter/Uniconta-PowerBI/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{43A97121-8B5A-4824-BB40-27EE5AA553E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0375D87-9E17-4FDB-ADC5-953DEFFFC0EE}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{43A97121-8B5A-4824-BB40-27EE5AA553E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A63BC79-0A23-4138-A854-4DCD03EE39C0}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{ED6A3BE0-DE88-465A-973D-FB8D93E934E7}"/>
   </bookViews>
   <sheets>
-    <sheet name="Egne labels" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -634,6 +634,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>